<commit_message>
feat(ui): droplists com busca e selecao multipla, slider duplo de nota, ordenacao decrescente e logo oficial
</commit_message>
<xml_diff>
--- a/docs/relatorios/geral.xlsx
+++ b/docs/relatorios/geral.xlsx
@@ -583,40 +583,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Acre</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>15</v>
       </c>
       <c r="D2" t="n">
-        <v>13.5</v>
+        <v>15</v>
       </c>
       <c r="E2" t="n">
-        <v>11.5</v>
+        <v>15</v>
       </c>
       <c r="F2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I2" t="n">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="J2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -627,40 +627,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alagoas</t>
+          <t>Espírito Santo — Polícia Penal</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>15</v>
       </c>
       <c r="D3" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H3" t="n">
-        <v>14.5</v>
+        <v>25</v>
       </c>
       <c r="I3" t="n">
-        <v>68.5</v>
+        <v>100</v>
       </c>
       <c r="J3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>74.5</v>
+        <v>100</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -671,12 +671,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Goiás</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -689,22 +689,22 @@
         <v>15</v>
       </c>
       <c r="F4" t="n">
-        <v>13.5</v>
+        <v>15</v>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I4" t="n">
-        <v>85.5</v>
+        <v>100</v>
       </c>
       <c r="J4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>91.5</v>
+        <v>100</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -759,12 +759,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -777,22 +777,22 @@
         <v>15</v>
       </c>
       <c r="F6" t="n">
-        <v>11.5</v>
+        <v>15</v>
       </c>
       <c r="G6" t="n">
         <v>15</v>
       </c>
       <c r="H6" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I6" t="n">
-        <v>88.5</v>
+        <v>96</v>
       </c>
       <c r="J6" t="n">
         <v>4</v>
       </c>
       <c r="K6" t="n">
-        <v>92.5</v>
+        <v>100</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -803,12 +803,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Roraima</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -818,10 +818,10 @@
         <v>15</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>11.5</v>
       </c>
       <c r="F7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G7" t="n">
         <v>15</v>
@@ -830,10 +830,10 @@
         <v>25</v>
       </c>
       <c r="I7" t="n">
-        <v>100</v>
+        <v>94.5</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="K7" t="n">
         <v>100</v>
@@ -847,12 +847,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Distrito Federal</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -865,7 +865,7 @@
         <v>15</v>
       </c>
       <c r="F8" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="G8" t="n">
         <v>15</v>
@@ -874,13 +874,13 @@
         <v>25</v>
       </c>
       <c r="I8" t="n">
-        <v>90.5</v>
+        <v>92.5</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K8" t="n">
-        <v>93.5</v>
+        <v>98.5</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -891,12 +891,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Espírito Santo — Polícia Penal</t>
+          <t>Mato Grosso</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -909,22 +909,22 @@
         <v>15</v>
       </c>
       <c r="F9" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G9" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H9" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="I9" t="n">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K9" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -935,12 +935,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Espírito Santo — SEJUS/ES</t>
+          <t>Minas Gerais</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -950,25 +950,25 @@
         <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>7.5</v>
+        <v>15</v>
       </c>
       <c r="F10" t="n">
-        <v>8</v>
+        <v>13.5</v>
       </c>
       <c r="G10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H10" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I10" t="n">
-        <v>80.5</v>
+        <v>90.5</v>
       </c>
       <c r="J10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>84.5</v>
+        <v>95.5</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -979,19 +979,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Goiás</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>15</v>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E11" t="n">
         <v>15</v>
@@ -1003,16 +1003,16 @@
         <v>15</v>
       </c>
       <c r="H11" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I11" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K11" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -1023,56 +1023,56 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Maranhão</t>
+          <t>Acre</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>15</v>
       </c>
       <c r="D12" t="n">
-        <v>15</v>
+        <v>13.5</v>
       </c>
       <c r="E12" t="n">
-        <v>15</v>
+        <v>11.5</v>
       </c>
       <c r="F12" t="n">
         <v>13</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H12" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I12" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J12" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K12" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Instituída — abaixo do mínimo em dimensão essencial</t>
+          <t>Instituída — seguindo os parâmetros mínimos</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mato Grosso</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1082,25 +1082,25 @@
         <v>15</v>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>11.5</v>
       </c>
       <c r="F13" t="n">
-        <v>13</v>
+        <v>11.5</v>
       </c>
       <c r="G13" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H13" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I13" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="J13" t="n">
         <v>10</v>
       </c>
       <c r="K13" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1111,12 +1111,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mato Grosso do Sul</t>
+          <t>Distrito Federal</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1126,25 +1126,25 @@
         <v>12</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F14" t="n">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="G14" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I14" t="n">
-        <v>78.5</v>
+        <v>90.5</v>
       </c>
       <c r="J14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>87.5</v>
+        <v>93.5</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1155,12 +1155,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Minas Gerais</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1173,7 +1173,7 @@
         <v>15</v>
       </c>
       <c r="F15" t="n">
-        <v>13.5</v>
+        <v>11.5</v>
       </c>
       <c r="G15" t="n">
         <v>15</v>
@@ -1182,13 +1182,13 @@
         <v>17</v>
       </c>
       <c r="I15" t="n">
-        <v>90.5</v>
+        <v>88.5</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K15" t="n">
-        <v>95.5</v>
+        <v>92.5</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1199,135 +1199,144 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pará</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>13.5</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="I16" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="J16" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" t="n">
+        <v>91.5</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Não instituída</t>
+          <t>Instituída — seguindo os parâmetros mínimos</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Paraíba</t>
+          <t>Pernambuco</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>15</v>
       </c>
       <c r="D17" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>15</v>
+        <v>10.5</v>
       </c>
       <c r="G17" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H17" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I17" t="n">
-        <v>79</v>
+        <v>85.5</v>
       </c>
       <c r="J17" t="n">
         <v>6</v>
       </c>
       <c r="K17" t="n">
-        <v>85</v>
+        <v>91.5</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Instituída — abaixo do mínimo em dimensão essencial</t>
+          <t>Instituída — seguindo os parâmetros mínimos</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Maranhão</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>15</v>
       </c>
       <c r="D18" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E18" t="n">
         <v>15</v>
       </c>
       <c r="F18" t="n">
-        <v>10.5</v>
+        <v>13</v>
       </c>
       <c r="G18" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="H18" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="I18" t="n">
-        <v>92.5</v>
+        <v>84</v>
       </c>
       <c r="J18" t="n">
         <v>6</v>
       </c>
       <c r="K18" t="n">
-        <v>98.5</v>
+        <v>90</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Instituída — seguindo os parâmetros mínimos</t>
+          <t>Instituída — abaixo do mínimo em dimensão essencial</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Pernambuco</t>
+          <t>Rio Grande do Sul</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1337,25 +1346,25 @@
         <v>12</v>
       </c>
       <c r="E19" t="n">
-        <v>15</v>
+        <v>11.5</v>
       </c>
       <c r="F19" t="n">
-        <v>10.5</v>
+        <v>13</v>
       </c>
       <c r="G19" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H19" t="n">
-        <v>23</v>
+        <v>16.5</v>
       </c>
       <c r="I19" t="n">
-        <v>85.5</v>
+        <v>83</v>
       </c>
       <c r="J19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K19" t="n">
-        <v>91.5</v>
+        <v>88</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1366,100 +1375,100 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Mato Grosso do Sul</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>15</v>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E20" t="n">
-        <v>11.5</v>
+        <v>8</v>
       </c>
       <c r="F20" t="n">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="G20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H20" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="I20" t="n">
-        <v>73</v>
+        <v>78.5</v>
       </c>
       <c r="J20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K20" t="n">
-        <v>80</v>
+        <v>87.5</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Instituída — abaixo do mínimo em dimensão essencial</t>
+          <t>Instituída — seguindo os parâmetros mínimos</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
+          <t>Paraíba</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>15</v>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E21" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
         <v>15</v>
       </c>
       <c r="G21" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="H21" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I21" t="n">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="J21" t="n">
         <v>6</v>
       </c>
       <c r="K21" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Instituída — seguindo os parâmetros mínimos</t>
+          <t>Instituída — abaixo do mínimo em dimensão essencial</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Espírito Santo — SEJUS/ES</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1469,25 +1478,25 @@
         <v>15</v>
       </c>
       <c r="E22" t="n">
-        <v>11.5</v>
+        <v>7.5</v>
       </c>
       <c r="F22" t="n">
-        <v>11.5</v>
+        <v>8</v>
       </c>
       <c r="G22" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H22" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I22" t="n">
-        <v>85</v>
+        <v>80.5</v>
       </c>
       <c r="J22" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K22" t="n">
-        <v>95</v>
+        <v>84.5</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1498,119 +1507,128 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Rio Grande do Sul</t>
+          <t>Santa Catarina</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>15</v>
       </c>
       <c r="D23" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E23" t="n">
-        <v>11.5</v>
+        <v>15</v>
       </c>
       <c r="F23" t="n">
-        <v>13</v>
+        <v>13.5</v>
       </c>
       <c r="G23" t="n">
         <v>15</v>
       </c>
       <c r="H23" t="n">
-        <v>16.5</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>83</v>
+        <v>77.5</v>
       </c>
       <c r="J23" t="n">
         <v>5</v>
       </c>
       <c r="K23" t="n">
-        <v>88</v>
+        <v>82.5</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Instituída — seguindo os parâmetros mínimos</t>
+          <t>Instituída — abaixo do mínimo em dimensão essencial</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Piauí</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>9.5</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="I24" t="n">
+        <v>73</v>
+      </c>
+      <c r="J24" t="n">
+        <v>7</v>
+      </c>
+      <c r="K24" t="n">
+        <v>80</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Não instituída</t>
+          <t>Instituída — abaixo do mínimo em dimensão essencial</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Roraima</t>
+          <t>Alagoas</t>
         </is>
       </c>
       <c r="C25" t="n">
         <v>15</v>
       </c>
       <c r="D25" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E25" t="n">
-        <v>11.5</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G25" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H25" t="n">
-        <v>25</v>
+        <v>14.5</v>
       </c>
       <c r="I25" t="n">
-        <v>94.5</v>
+        <v>68.5</v>
       </c>
       <c r="J25" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="K25" t="n">
-        <v>100</v>
+        <v>74.5</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1621,40 +1639,40 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Santa Catarina</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>15</v>
       </c>
       <c r="D26" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>13.5</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>77.5</v>
+        <v>15</v>
       </c>
       <c r="J26" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>82.5</v>
+        <v>15</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1665,60 +1683,51 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Pará</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>21</v>
-      </c>
-      <c r="I27" t="n">
-        <v>96</v>
-      </c>
-      <c r="J27" t="n">
-        <v>4</v>
-      </c>
-      <c r="K27" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Instituída — seguindo os parâmetros mínimos</t>
+          <t>Não instituída</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Rondônia</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -1727,7 +1736,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1735,18 +1744,9 @@
       <c r="H28" t="n">
         <v>0</v>
       </c>
-      <c r="I28" t="n">
-        <v>15</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>15</v>
-      </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Instituída — abaixo do mínimo em dimensão essencial</t>
+          <t>Não instituída</t>
         </is>
       </c>
     </row>

</xml_diff>